<commit_message>
Agrega luces nocturnas VIIRS 2012-2024 por distrito
Compuestos anuales VNL V2 (copia abierta en Zenodo, CC BY 4.0) recortados
a Paraguay y armonizados a nW/cm²/sr: la copia trae 2012-2021
multiplicado por 10. Suma, media y % de píxeles iluminados por distrito
y año, calculados con los límites COD-AB de OCHA (263 distritos,
incluidos los 13 nuevos de 2022). Se agregan las columnas luz_* a la base
distrital sin modificar las existentes, y se actualizan diccionario,
catálogo, fuentes_maestro (F049), arquitectura, README e inventario.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UUJkAC8tnPcgu9dLUHT9pp
</commit_message>
<xml_diff>
--- a/catalogo_bases_caminos_vecinales.xlsx
+++ b/catalogo_bases_caminos_vecinales.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Pedidos sugeridos" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Catálogo!$A$1:$P$42</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Catálogo!$A$1:$P$43</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="527">
   <si>
     <t xml:space="preserve">Catálogo y repositorio de datos – Caminos vecinales y condiciones de vida rural (v2)</t>
   </si>
@@ -1492,6 +1492,42 @@
   </si>
   <si>
     <t xml:space="preserve">Mapas rápidos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luces nocturnas VIIRS anuales (VNL V2) 2012-2024 – recorte Paraguay y suma por distrito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payne Institute / EOG (Colorado School of Mines), copia en Zenodo (T. Hengl)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compuestos anuales de radiancia nocturna a 500 m, recortados a Paraguay, más una tabla con suma, media y % de píxeles iluminados por distrito y año.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">luz_suma, luz_media, pct_pixeles_iluminados por distrito (263) y año (2012-2024).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Píxel 500 m; distrito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2012-2024 (anual)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GeoTIFF (13) + CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://zenodo.org/records/17294744</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultado anual por distrito (actividad económica / electrificación): es la variable que hace posible el diseño de diferencias en diferencias escalonado. En los distritos foco, la luz por habitante 2022 se correlaciona con el IPM rural (ρ = −0,48).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La copia de Zenodo guarda 2012-2021 multiplicado por 10 y 2022-2024 sin multiplicar: se armonizó a nW/cm²/sr. Valores enteros (precisión 1 nW): la luz rural muy tenue queda en 0. 2012 cubre abr-dic. Hay píxeles atípicos (incendios) en 2012 y 2018. Para más precisión, bajar el producto original (decimal) con una cuenta gratuita en eogdata.mines.edu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07_clima_y_contexto/luces_nocturnas_VIIRS</t>
   </si>
   <si>
     <t xml:space="preserve">Qué pedir</t>
@@ -1759,8 +1795,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1828,7 +1868,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2188,214 +2228,214 @@
   <dimension ref="A1:B28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="105"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="B1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4"/>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4"/>
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <f aca="false">COUNTIF(Catálogo!N:N,"Descargado y procesado")</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <f aca="false">COUNTIF(Catálogo!N:N,"Descargado")</f>
         <v>25</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <f aca="false">COUNTIF(Catálogo!N:N,"Parcial")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <f aca="false">COUNTIF(Catálogo!N:N,"Requiere pedido")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <f aca="false">COUNTIF(Catálogo!N:N,"No disponible")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <f aca="false">COUNTIF(Catálogo!N:N,"En línea (no descargable)")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="3" t="n">
         <f aca="false">COUNTA(Catálogo!A:A)-1</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="2"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3"/>
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="3"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="B25" s="3"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2415,2023 +2455,2071 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="28"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+    <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="N2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="P2" s="10"/>
-    </row>
-    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="P2" s="11"/>
+    </row>
+    <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="L3" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="M3" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="N3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="O3" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="P3" s="10"/>
-    </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="P3" s="11"/>
+    </row>
+    <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="J4" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="N4" s="8" t="s">
+      <c r="N4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O4" s="6" t="s">
+      <c r="O4" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="P4" s="10"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="P4" s="11"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J5" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L5" s="6" t="s">
+      <c r="L5" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="M5" s="6" t="s">
+      <c r="M5" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="N5" s="8" t="s">
+      <c r="N5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="P5" s="10"/>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="P5" s="11"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="K6" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="L6" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="N6" s="8" t="s">
+      <c r="N6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O6" s="6" t="s">
+      <c r="O6" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="P6" s="10"/>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="P6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="K7" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L7" s="6" t="s">
+      <c r="L7" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="M7" s="6" t="s">
+      <c r="M7" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="N7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="6" t="s">
+      <c r="O7" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="P7" s="10"/>
-    </row>
-    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="P7" s="11"/>
+    </row>
+    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="L8" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="M8" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="N8" s="9" t="s">
+      <c r="N8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O8" s="6" t="s">
+      <c r="O8" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="P8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="P8" s="11"/>
+    </row>
+    <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="K9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="M9" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="O9" s="6" t="s">
+      <c r="O9" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="P9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="P9" s="11"/>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="I10" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="K10" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="L10" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="M10" s="6"/>
-      <c r="N10" s="8" t="s">
+      <c r="M10" s="7"/>
+      <c r="N10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O10" s="6" t="s">
+      <c r="O10" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="P10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="P10" s="11"/>
+    </row>
+    <row r="11" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="J11" s="11" t="s">
+      <c r="J11" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="K11" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L11" s="6" t="s">
+      <c r="L11" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="M11" s="6" t="s">
+      <c r="M11" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="N11" s="8" t="s">
+      <c r="N11" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O11" s="6" t="s">
+      <c r="O11" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="P11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="P11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="K12" s="12" t="s">
+      <c r="K12" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L12" s="6" t="s">
+      <c r="L12" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="M12" s="6"/>
-      <c r="N12" s="8" t="s">
+      <c r="M12" s="7"/>
+      <c r="N12" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O12" s="6" t="s">
+      <c r="O12" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="P12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="P12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="K13" s="12" t="s">
+      <c r="K13" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L13" s="6" t="s">
+      <c r="L13" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="M13" s="6" t="s">
+      <c r="M13" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="N13" s="13" t="s">
+      <c r="N13" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="O13" s="6"/>
-      <c r="P13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="O13" s="7"/>
+      <c r="P13" s="11"/>
+    </row>
+    <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="H14" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="J14" s="11" t="s">
+      <c r="J14" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="K14" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L14" s="6" t="s">
+      <c r="L14" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="M14" s="6" t="s">
+      <c r="M14" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="N14" s="9" t="s">
+      <c r="N14" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O14" s="6" t="s">
+      <c r="O14" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="P14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="P14" s="11"/>
+    </row>
+    <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G15" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="H15" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="I15" s="6" t="s">
+      <c r="I15" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="K15" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L15" s="6" t="s">
+      <c r="L15" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="M15" s="6" t="s">
+      <c r="M15" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="N15" s="8" t="s">
+      <c r="N15" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O15" s="6" t="s">
+      <c r="O15" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="P15" s="10"/>
-    </row>
-    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="P15" s="11"/>
+    </row>
+    <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="G16" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="H16" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="I16" s="6" t="s">
+      <c r="I16" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="K16" s="12" t="s">
+      <c r="K16" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L16" s="6" t="s">
+      <c r="L16" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="M16" s="6" t="s">
+      <c r="M16" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="N16" s="8" t="s">
+      <c r="N16" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O16" s="6" t="s">
+      <c r="O16" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="P16" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="P16" s="11"/>
+    </row>
+    <row r="17" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="J17" s="11" t="s">
+      <c r="J17" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="K17" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L17" s="6" t="s">
+      <c r="L17" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="M17" s="6" t="s">
+      <c r="M17" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="N17" s="9" t="s">
+      <c r="N17" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O17" s="6" t="s">
+      <c r="O17" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="P17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="P17" s="11"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="H18" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="I18" s="6" t="s">
+      <c r="I18" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="J18" s="11" t="s">
+      <c r="J18" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="K18" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L18" s="6" t="s">
+      <c r="L18" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="M18" s="6" t="s">
+      <c r="M18" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="N18" s="14" t="s">
+      <c r="N18" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="O18" s="6"/>
-      <c r="P18" s="10"/>
-    </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="O18" s="7"/>
+      <c r="P18" s="11"/>
+    </row>
+    <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="11" t="s">
+      <c r="J19" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="K19" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="L19" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="M19" s="6" t="s">
+      <c r="M19" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="N19" s="9" t="s">
+      <c r="N19" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O19" s="6" t="s">
+      <c r="O19" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="P19" s="10"/>
-    </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="P19" s="11"/>
+    </row>
+    <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G20" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="H20" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="J20" s="11" t="s">
+      <c r="J20" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="K20" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="L20" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="M20" s="6" t="s">
+      <c r="M20" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="N20" s="8" t="s">
+      <c r="N20" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O20" s="6" t="s">
+      <c r="O20" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="P20" s="10"/>
-    </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="P20" s="11"/>
+    </row>
+    <row r="21" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="I21" s="7" t="s">
         <v>258</v>
       </c>
-      <c r="J21" s="11" t="s">
+      <c r="J21" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="K21" s="12" t="s">
+      <c r="K21" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="M21" s="6" t="s">
+      <c r="M21" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="N21" s="8" t="s">
+      <c r="N21" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O21" s="6" t="s">
+      <c r="O21" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="P21" s="10"/>
-    </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="P21" s="11"/>
+    </row>
+    <row r="22" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G22" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="H22" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="J22" s="11" t="s">
+      <c r="J22" s="12" t="s">
         <v>270</v>
       </c>
-      <c r="K22" s="8" t="s">
+      <c r="K22" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="L22" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="M22" s="6" t="s">
+      <c r="M22" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="N22" s="8" t="s">
+      <c r="N22" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O22" s="6" t="s">
+      <c r="O22" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="P22" s="10"/>
-    </row>
-    <row r="23" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="P22" s="11"/>
+    </row>
+    <row r="23" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="7" t="s">
         <v>278</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>280</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="J23" s="11" t="s">
+      <c r="J23" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="K23" s="12" t="s">
+      <c r="K23" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L23" s="6" t="s">
+      <c r="L23" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="M23" s="6" t="s">
+      <c r="M23" s="7" t="s">
         <v>284</v>
       </c>
-      <c r="N23" s="9" t="s">
+      <c r="N23" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O23" s="6" t="s">
+      <c r="O23" s="7" t="s">
         <v>285</v>
       </c>
-      <c r="P23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="P23" s="11"/>
+    </row>
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="7" t="s">
         <v>288</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="H24" s="7" t="s">
         <v>291</v>
       </c>
-      <c r="I24" s="6" t="s">
+      <c r="I24" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="J24" s="11" t="s">
+      <c r="J24" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="K24" s="15" t="s">
+      <c r="K24" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="L24" s="6" t="s">
+      <c r="L24" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="M24" s="6" t="s">
+      <c r="M24" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="N24" s="8" t="s">
+      <c r="N24" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O24" s="6" t="s">
+      <c r="O24" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="P24" s="10"/>
-    </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
+      <c r="P24" s="11"/>
+    </row>
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F25" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="G25" s="6" t="s">
+      <c r="G25" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="H25" s="6" t="s">
+      <c r="H25" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="I25" s="6" t="s">
+      <c r="I25" s="7" t="s">
         <v>304</v>
       </c>
-      <c r="J25" s="11" t="s">
+      <c r="J25" s="12" t="s">
         <v>305</v>
       </c>
-      <c r="K25" s="15" t="s">
+      <c r="K25" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="M25" s="6" t="s">
+      <c r="M25" s="7" t="s">
         <v>307</v>
       </c>
-      <c r="N25" s="13" t="s">
+      <c r="N25" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="O25" s="6"/>
-      <c r="P25" s="10"/>
-    </row>
-    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
+      <c r="O25" s="7"/>
+      <c r="P25" s="11"/>
+    </row>
+    <row r="26" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="7" t="s">
         <v>311</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" s="7" t="s">
         <v>312</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="G26" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="H26" s="6" t="s">
+      <c r="H26" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="I26" s="6" t="s">
+      <c r="I26" s="7" t="s">
         <v>314</v>
       </c>
-      <c r="J26" s="11" t="s">
+      <c r="J26" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="K26" s="8" t="s">
+      <c r="K26" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L26" s="6" t="s">
+      <c r="L26" s="7" t="s">
         <v>316</v>
       </c>
-      <c r="M26" s="6" t="s">
+      <c r="M26" s="7" t="s">
         <v>317</v>
       </c>
-      <c r="N26" s="8" t="s">
+      <c r="N26" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O26" s="6" t="s">
+      <c r="O26" s="7" t="s">
         <v>318</v>
       </c>
-      <c r="P26" s="10"/>
-    </row>
-    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="P26" s="11"/>
+    </row>
+    <row r="27" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="7" t="s">
         <v>323</v>
       </c>
-      <c r="G27" s="6" t="s">
+      <c r="G27" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="H27" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="I27" s="6" t="s">
+      <c r="I27" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="J27" s="11" t="s">
+      <c r="J27" s="12" t="s">
         <v>327</v>
       </c>
-      <c r="K27" s="8" t="s">
+      <c r="K27" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L27" s="6" t="s">
+      <c r="L27" s="7" t="s">
         <v>328</v>
       </c>
-      <c r="M27" s="6" t="s">
+      <c r="M27" s="7" t="s">
         <v>329</v>
       </c>
-      <c r="N27" s="8" t="s">
+      <c r="N27" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O27" s="6" t="s">
+      <c r="O27" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="P27" s="10"/>
-    </row>
-    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+      <c r="P27" s="11"/>
+    </row>
+    <row r="28" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
         <v>331</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>332</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="7" t="s">
         <v>334</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F28" s="7" t="s">
         <v>335</v>
       </c>
-      <c r="G28" s="6" t="s">
+      <c r="G28" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="H28" s="6" t="s">
+      <c r="H28" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="I28" s="6" t="s">
+      <c r="I28" s="7" t="s">
         <v>336</v>
       </c>
-      <c r="J28" s="11" t="s">
+      <c r="J28" s="12" t="s">
         <v>337</v>
       </c>
-      <c r="K28" s="8" t="s">
+      <c r="K28" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L28" s="6" t="s">
+      <c r="L28" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="M28" s="6" t="s">
+      <c r="M28" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="N28" s="16" t="s">
+      <c r="N28" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="O28" s="6"/>
-      <c r="P28" s="10"/>
-    </row>
-    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
+      <c r="O28" s="7"/>
+      <c r="P28" s="11"/>
+    </row>
+    <row r="29" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
         <v>340</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>341</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>342</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="7" t="s">
         <v>343</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="7" t="s">
         <v>344</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="G29" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="H29" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="I29" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="J29" s="11" t="s">
+      <c r="J29" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="K29" s="12" t="s">
+      <c r="K29" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L29" s="6" t="s">
+      <c r="L29" s="7" t="s">
         <v>347</v>
       </c>
-      <c r="M29" s="6" t="s">
+      <c r="M29" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="N29" s="8" t="s">
+      <c r="N29" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O29" s="6" t="s">
+      <c r="O29" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="P29" s="10"/>
-    </row>
-    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
+      <c r="P29" s="11"/>
+    </row>
+    <row r="30" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
         <v>350</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>351</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="7" t="s">
         <v>353</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="7" t="s">
         <v>354</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F30" s="7" t="s">
         <v>355</v>
       </c>
-      <c r="G30" s="6" t="s">
+      <c r="G30" s="7" t="s">
         <v>356</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="H30" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="I30" s="6" t="s">
+      <c r="I30" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="J30" s="11" t="s">
+      <c r="J30" s="12" t="s">
         <v>358</v>
       </c>
-      <c r="K30" s="8" t="s">
+      <c r="K30" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L30" s="6" t="s">
+      <c r="L30" s="7" t="s">
         <v>359</v>
       </c>
-      <c r="M30" s="6" t="s">
+      <c r="M30" s="7" t="s">
         <v>360</v>
       </c>
-      <c r="N30" s="8" t="s">
+      <c r="N30" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O30" s="6" t="s">
+      <c r="O30" s="7" t="s">
         <v>361</v>
       </c>
-      <c r="P30" s="10"/>
-    </row>
-    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="P30" s="11"/>
+    </row>
+    <row r="31" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
         <v>362</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>351</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="7" t="s">
         <v>364</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="7" t="s">
         <v>365</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="F31" s="7" t="s">
         <v>366</v>
       </c>
-      <c r="G31" s="6" t="s">
+      <c r="G31" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="H31" s="6" t="s">
+      <c r="H31" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="I31" s="6" t="s">
+      <c r="I31" s="7" t="s">
         <v>368</v>
       </c>
-      <c r="J31" s="11" t="s">
+      <c r="J31" s="12" t="s">
         <v>369</v>
       </c>
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L31" s="6" t="s">
+      <c r="L31" s="7" t="s">
         <v>370</v>
       </c>
-      <c r="M31" s="6"/>
-      <c r="N31" s="8" t="s">
+      <c r="M31" s="7"/>
+      <c r="N31" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O31" s="6" t="s">
+      <c r="O31" s="7" t="s">
         <v>371</v>
       </c>
-      <c r="P31" s="10"/>
-    </row>
-    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+      <c r="P31" s="11"/>
+    </row>
+    <row r="32" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
         <v>372</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="8" t="s">
         <v>374</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="7" t="s">
         <v>375</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="7" t="s">
         <v>376</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="7" t="s">
         <v>377</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="I32" s="6" t="s">
+      <c r="I32" s="7" t="s">
         <v>379</v>
       </c>
-      <c r="J32" s="11" t="s">
+      <c r="J32" s="12" t="s">
         <v>380</v>
       </c>
-      <c r="K32" s="8" t="s">
+      <c r="K32" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="7" t="s">
         <v>381</v>
       </c>
-      <c r="M32" s="6" t="s">
+      <c r="M32" s="7" t="s">
         <v>382</v>
       </c>
-      <c r="N32" s="8" t="s">
+      <c r="N32" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O32" s="6" t="s">
+      <c r="O32" s="7" t="s">
         <v>383</v>
       </c>
-      <c r="P32" s="10"/>
-    </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
+      <c r="P32" s="11"/>
+    </row>
+    <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
         <v>384</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="8" t="s">
         <v>385</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="7" t="s">
         <v>386</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="7" t="s">
         <v>387</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="F33" s="7" t="s">
         <v>388</v>
       </c>
-      <c r="G33" s="6" t="s">
+      <c r="G33" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="H33" s="7" t="s">
         <v>390</v>
       </c>
-      <c r="I33" s="6" t="s">
+      <c r="I33" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="J33" s="11" t="s">
+      <c r="J33" s="12" t="s">
         <v>391</v>
       </c>
-      <c r="K33" s="12" t="s">
+      <c r="K33" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L33" s="6" t="s">
+      <c r="L33" s="7" t="s">
         <v>392</v>
       </c>
-      <c r="M33" s="6" t="s">
+      <c r="M33" s="7" t="s">
         <v>393</v>
       </c>
-      <c r="N33" s="8" t="s">
+      <c r="N33" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O33" s="6" t="s">
+      <c r="O33" s="7" t="s">
         <v>394</v>
       </c>
-      <c r="P33" s="10"/>
-    </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
+      <c r="P33" s="11"/>
+    </row>
+    <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="8" t="s">
         <v>396</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="F34" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="G34" s="6" t="s">
+      <c r="G34" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="H34" s="6" t="s">
+      <c r="H34" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="I34" s="6" t="s">
+      <c r="I34" s="7" t="s">
         <v>402</v>
       </c>
-      <c r="J34" s="11" t="s">
+      <c r="J34" s="12" t="s">
         <v>403</v>
       </c>
-      <c r="K34" s="12" t="s">
+      <c r="K34" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L34" s="6" t="s">
+      <c r="L34" s="7" t="s">
         <v>404</v>
       </c>
-      <c r="M34" s="6" t="s">
+      <c r="M34" s="7" t="s">
         <v>405</v>
       </c>
-      <c r="N34" s="8" t="s">
+      <c r="N34" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O34" s="6" t="s">
+      <c r="O34" s="7" t="s">
         <v>406</v>
       </c>
-      <c r="P34" s="10"/>
-    </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
+      <c r="P34" s="11"/>
+    </row>
+    <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
         <v>407</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="F35" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="G35" s="6" t="s">
+      <c r="G35" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="H35" s="6" t="s">
+      <c r="H35" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="I35" s="6" t="s">
+      <c r="I35" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="J35" s="11" t="s">
+      <c r="J35" s="12" t="s">
         <v>415</v>
       </c>
-      <c r="K35" s="15" t="s">
+      <c r="K35" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="L35" s="6" t="s">
+      <c r="L35" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="M35" s="6" t="s">
+      <c r="M35" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="N35" s="14" t="s">
+      <c r="N35" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="O35" s="6"/>
-      <c r="P35" s="10"/>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
+      <c r="O35" s="7"/>
+      <c r="P35" s="11"/>
+    </row>
+    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="8" t="s">
         <v>420</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="7" t="s">
         <v>422</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="F36" s="7" t="s">
         <v>423</v>
       </c>
-      <c r="G36" s="6" t="s">
+      <c r="G36" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="H36" s="6" t="s">
+      <c r="H36" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="I36" s="6" t="s">
+      <c r="I36" s="7" t="s">
         <v>426</v>
       </c>
-      <c r="J36" s="11" t="s">
+      <c r="J36" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="K36" s="8" t="s">
+      <c r="K36" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L36" s="6" t="s">
+      <c r="L36" s="7" t="s">
         <v>428</v>
       </c>
-      <c r="M36" s="6" t="s">
+      <c r="M36" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="N36" s="16" t="s">
+      <c r="N36" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="O36" s="6"/>
-      <c r="P36" s="10"/>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+      <c r="O36" s="7"/>
+      <c r="P36" s="11"/>
+    </row>
+    <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
         <v>430</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="8" t="s">
         <v>431</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="7" t="s">
         <v>432</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" s="7" t="s">
         <v>433</v>
       </c>
-      <c r="F37" s="6" t="s">
+      <c r="F37" s="7" t="s">
         <v>434</v>
       </c>
-      <c r="G37" s="6" t="s">
+      <c r="G37" s="7" t="s">
         <v>435</v>
       </c>
-      <c r="H37" s="6" t="s">
+      <c r="H37" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="I37" s="6" t="s">
+      <c r="I37" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="J37" s="11" t="s">
+      <c r="J37" s="12" t="s">
         <v>436</v>
       </c>
-      <c r="K37" s="8" t="s">
+      <c r="K37" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L37" s="6" t="s">
+      <c r="L37" s="7" t="s">
         <v>437</v>
       </c>
-      <c r="M37" s="6" t="s">
+      <c r="M37" s="7" t="s">
         <v>438</v>
       </c>
-      <c r="N37" s="16" t="s">
+      <c r="N37" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="O37" s="6"/>
-      <c r="P37" s="10"/>
-    </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+      <c r="O37" s="7"/>
+      <c r="P37" s="11"/>
+    </row>
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
         <v>439</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="8" t="s">
         <v>440</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="E38" s="7" t="s">
         <v>441</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="F38" s="7" t="s">
         <v>442</v>
       </c>
-      <c r="G38" s="6" t="s">
+      <c r="G38" s="7" t="s">
         <v>443</v>
       </c>
-      <c r="H38" s="6" t="s">
+      <c r="H38" s="7" t="s">
         <v>444</v>
       </c>
-      <c r="I38" s="6" t="s">
+      <c r="I38" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="J38" s="11" t="s">
+      <c r="J38" s="12" t="s">
         <v>445</v>
       </c>
-      <c r="K38" s="15" t="s">
+      <c r="K38" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="L38" s="6" t="s">
+      <c r="L38" s="7" t="s">
         <v>446</v>
       </c>
-      <c r="M38" s="6" t="s">
+      <c r="M38" s="7" t="s">
         <v>447</v>
       </c>
-      <c r="N38" s="13" t="s">
+      <c r="N38" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="O38" s="6"/>
-      <c r="P38" s="10"/>
-    </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
+      <c r="O38" s="7"/>
+      <c r="P38" s="11"/>
+    </row>
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
         <v>448</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="8" t="s">
         <v>450</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="E39" s="7" t="s">
         <v>451</v>
       </c>
-      <c r="F39" s="6" t="s">
+      <c r="F39" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="G39" s="6" t="s">
+      <c r="G39" s="7" t="s">
         <v>453</v>
       </c>
-      <c r="H39" s="6" t="s">
+      <c r="H39" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="I39" s="6" t="s">
+      <c r="I39" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="J39" s="11" t="s">
+      <c r="J39" s="12" t="s">
         <v>455</v>
       </c>
-      <c r="K39" s="8" t="s">
+      <c r="K39" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L39" s="6" t="s">
+      <c r="L39" s="7" t="s">
         <v>456</v>
       </c>
-      <c r="M39" s="6" t="s">
+      <c r="M39" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="N39" s="8" t="s">
+      <c r="N39" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O39" s="6" t="s">
+      <c r="O39" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="P39" s="10"/>
-    </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
+      <c r="P39" s="11"/>
+    </row>
+    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
         <v>459</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="8" t="s">
         <v>460</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D40" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="E40" s="7" t="s">
         <v>461</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="F40" s="7" t="s">
         <v>462</v>
       </c>
-      <c r="G40" s="6" t="s">
+      <c r="G40" s="7" t="s">
         <v>463</v>
       </c>
-      <c r="H40" s="6" t="s">
+      <c r="H40" s="7" t="s">
         <v>464</v>
       </c>
-      <c r="I40" s="6" t="s">
+      <c r="I40" s="7" t="s">
         <v>465</v>
       </c>
-      <c r="J40" s="11" t="s">
+      <c r="J40" s="12" t="s">
         <v>466</v>
       </c>
-      <c r="K40" s="8" t="s">
+      <c r="K40" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L40" s="6" t="s">
+      <c r="L40" s="7" t="s">
         <v>467</v>
       </c>
-      <c r="M40" s="6" t="s">
+      <c r="M40" s="7" t="s">
         <v>468</v>
       </c>
-      <c r="N40" s="8" t="s">
+      <c r="N40" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O40" s="6" t="s">
+      <c r="O40" s="7" t="s">
         <v>469</v>
       </c>
-      <c r="P40" s="10"/>
-    </row>
-    <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
+      <c r="P40" s="11"/>
+    </row>
+    <row r="41" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="8" t="s">
         <v>471</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D41" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="E41" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="F41" s="7" t="s">
         <v>474</v>
       </c>
-      <c r="G41" s="6" t="s">
+      <c r="G41" s="7" t="s">
         <v>475</v>
       </c>
-      <c r="H41" s="6" t="s">
+      <c r="H41" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="I41" s="7" t="s">
         <v>476</v>
       </c>
-      <c r="J41" s="11" t="s">
+      <c r="J41" s="12" t="s">
         <v>477</v>
       </c>
-      <c r="K41" s="12" t="s">
+      <c r="K41" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L41" s="6" t="s">
+      <c r="L41" s="7" t="s">
         <v>478</v>
       </c>
-      <c r="M41" s="6"/>
-      <c r="N41" s="8" t="s">
+      <c r="M41" s="7"/>
+      <c r="N41" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O41" s="6" t="s">
+      <c r="O41" s="7" t="s">
         <v>479</v>
       </c>
-      <c r="P41" s="10"/>
-    </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
+      <c r="P41" s="11"/>
+    </row>
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
         <v>480</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="8" t="s">
         <v>481</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="E42" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="F42" s="7" t="s">
         <v>483</v>
       </c>
-      <c r="G42" s="6" t="s">
+      <c r="G42" s="7" t="s">
         <v>484</v>
       </c>
-      <c r="H42" s="6" t="s">
+      <c r="H42" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="I42" s="6" t="s">
+      <c r="I42" s="7" t="s">
         <v>486</v>
       </c>
-      <c r="J42" s="11" t="s">
+      <c r="J42" s="12" t="s">
         <v>487</v>
       </c>
-      <c r="K42" s="12" t="s">
+      <c r="K42" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="L42" s="6" t="s">
+      <c r="L42" s="7" t="s">
         <v>488</v>
       </c>
-      <c r="M42" s="6"/>
-      <c r="N42" s="8" t="s">
+      <c r="M42" s="7"/>
+      <c r="N42" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O42" s="6" t="s">
+      <c r="O42" s="7" t="s">
         <v>469</v>
       </c>
-      <c r="P42" s="10"/>
+      <c r="P42" s="11"/>
+    </row>
+    <row r="43" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>490</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="I43" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="J43" s="12" t="s">
+        <v>497</v>
+      </c>
+      <c r="K43" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="L43" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="M43" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="N43" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="O43" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="P43" s="11"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P42"/>
+  <autoFilter ref="A1:P43"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N42" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N43" type="list">
       <formula1>"Descargado,Descargado y procesado,Parcial,Requiere pedido,No disponible,En línea (no descargable)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4476,6 +4564,7 @@
     <hyperlink ref="J40" r:id="rId37" display="https://www.ine.gov.py/microdatos/codigo-geografico-2022.php"/>
     <hyperlink ref="J41" r:id="rId38" display="https://data.humdata.org/dataset/cod-ab-pry"/>
     <hyperlink ref="J42" r:id="rId39" display="https://www.datos.gov.py/dataset/base-de-datos-geojson-geoespacial-de-departamentos-distritos-ciudades-y-barrios-de-todo-el"/>
+    <hyperlink ref="J43" r:id="rId40" display="https://zenodo.org/records/17294744"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4484,7 +4573,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId40"/>
+  <drawing r:id="rId41"/>
 </worksheet>
 </file>
 
@@ -4496,147 +4585,147 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="80"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="17" t="s">
-        <v>489</v>
-      </c>
-      <c r="C1" s="17" t="s">
-        <v>490</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>491</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+      <c r="B1" s="18" t="s">
+        <v>501</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>502</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>503</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>495</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
-        <v>497</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>498</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>499</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>500</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>501</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>503</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>500</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="B2" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>506</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>513</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>504</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>505</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>506</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="B5" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>517</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>518</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>507</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="B6" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>359</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
+        <v>520</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>508</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
         <v>421</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>509</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>510</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="B7" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>523</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>512</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>513</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>496</v>
+      <c r="B8" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>525</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>526</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>508</v>
       </c>
     </row>
   </sheetData>

</xml_diff>